<commit_message>
KHAZNA: IP55 coffrets supplied by SPIE, removed from FCI and memoir
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0139BLLtkKLWeHBxFoKLnQRG
</commit_message>
<xml_diff>
--- a/livrables/KHAZNA/Chiffrage/FCI_Khazna_CFA_SSI_AV_IT_v4.xlsx
+++ b/livrables/KHAZNA/Chiffrage/FCI_Khazna_CFA_SSI_AV_IT_v4.xlsx
@@ -667,7 +667,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>432.56</v>
+        <v>0</v>
       </c>
       <c r="F7" s="8">
         <f>D7*E7</f>
@@ -675,7 +675,7 @@
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>Fourniture Octet Plus devis DE044128 du 15/10/2026 (ZVK EasyLan, garantie système 25 ans ; baies LIEN'K), coffret 19" 12U étanche IP55 COF12645MIP55 (413,11 €) + bandeau 8 PC (19,45 €) = 432.56 €. Switch informatique fourni par EXYTE (pose et paramétrage PROSYB, MO à chiffrer). Tiroir optique compté dans la boucle fibre.</t>
+          <t>Coffret IP55 FOURNI ET POSÉ PAR SPIE (Ahmed, lot électricité) : retiré de l'offre et du devis Octet Plus DE044128 (COF12645MIP55 + bandeau). PROSYB installe dans ce coffret le tiroir optique et le panneau Cat. 6A (compatibilité 19"/rail DIN à valider avec SPIE). Switch informatique fourni par EXYTE (pose et paramétrage PROSYB, MO à chiffrer).</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>432.56</v>
+        <v>0</v>
       </c>
       <c r="F8" s="8">
         <f>D8*E8</f>
@@ -703,7 +703,7 @@
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
-          <t>Fourniture Octet Plus devis DE044128 du 15/10/2026 (ZVK EasyLan, garantie système 25 ans ; baies LIEN'K), coffret 19" 12U étanche IP55 COF12645MIP55 (413,11 €) + bandeau 8 PC (19,45 €) = 432.56 €. Switch informatique fourni par EXYTE (pose et paramétrage PROSYB, MO à chiffrer). Tiroir optique compté dans la boucle fibre.</t>
+          <t>Coffret IP55 FOURNI ET POSÉ PAR SPIE (Ahmed, lot électricité) : retiré de l'offre et du devis Octet Plus DE044128 (COF12645MIP55 + bandeau). PROSYB installe dans ce coffret le tiroir optique et le panneau Cat. 6A (compatibilité 19"/rail DIN à valider avec SPIE). Switch informatique fourni par EXYTE (pose et paramétrage PROSYB, MO à chiffrer).</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>432.56</v>
+        <v>0</v>
       </c>
       <c r="F9" s="8">
         <f>D9*E9</f>
@@ -731,7 +731,7 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Fourniture Octet Plus devis DE044128 du 15/10/2026 (ZVK EasyLan, garantie système 25 ans ; baies LIEN'K), coffret 19" 12U étanche IP55 COF12645MIP55 (413,11 €) + bandeau 8 PC (19,45 €) = 432.56 €. Switch informatique fourni par EXYTE (pose et paramétrage PROSYB, MO à chiffrer). Tiroir optique compté dans la boucle fibre.</t>
+          <t>Coffret IP55 FOURNI ET POSÉ PAR SPIE (Ahmed, lot électricité) : retiré de l'offre et du devis Octet Plus DE044128 (COF12645MIP55 + bandeau). PROSYB installe dans ce coffret le tiroir optique et le panneau Cat. 6A (compatibilité 19"/rail DIN à valider avec SPIE). Switch informatique fourni par EXYTE (pose et paramétrage PROSYB, MO à chiffrer).</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="11" t="n">
-        <v>432.56</v>
+        <v>0</v>
       </c>
       <c r="F10" s="8">
         <f>D10*E10</f>
@@ -759,7 +759,7 @@
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>Fourniture Octet Plus devis DE044128 du 15/10/2026 (ZVK EasyLan, garantie système 25 ans ; baies LIEN'K), coffret 19" 12U étanche IP55 COF12645MIP55 (413,11 €) + bandeau 8 PC (19,45 €) = 432.56 €. Switch informatique fourni par EXYTE (pose et paramétrage PROSYB, MO à chiffrer). Tiroir optique compté dans la boucle fibre.</t>
+          <t>Coffret IP55 FOURNI ET POSÉ PAR SPIE (Ahmed, lot électricité) : retiré de l'offre et du devis Octet Plus DE044128 (COF12645MIP55 + bandeau). PROSYB installe dans ce coffret le tiroir optique et le panneau Cat. 6A (compatibilité 19"/rail DIN à valider avec SPIE). Switch informatique fourni par EXYTE (pose et paramétrage PROSYB, MO à chiffrer).</t>
         </is>
       </c>
     </row>
@@ -779,7 +779,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="11" t="n">
-        <v>432.56</v>
+        <v>0</v>
       </c>
       <c r="F11" s="8">
         <f>D11*E11</f>
@@ -787,7 +787,7 @@
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>Fourniture Octet Plus devis DE044128 du 15/10/2026 (ZVK EasyLan, garantie système 25 ans ; baies LIEN'K), coffret 19" 12U étanche IP55 COF12645MIP55 (413,11 €) + bandeau 8 PC (19,45 €) = 432.56 €. Switch informatique fourni par EXYTE (pose et paramétrage PROSYB, MO à chiffrer). Tiroir optique compté dans la boucle fibre.</t>
+          <t>Coffret IP55 FOURNI ET POSÉ PAR SPIE (Ahmed, lot électricité) : retiré de l'offre et du devis Octet Plus DE044128 (COF12645MIP55 + bandeau). PROSYB installe dans ce coffret le tiroir optique et le panneau Cat. 6A (compatibilité 19"/rail DIN à valider avec SPIE). Switch informatique fourni par EXYTE (pose et paramétrage PROSYB, MO à chiffrer).</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
         <v>2</v>
       </c>
       <c r="E30" s="11" t="n">
-        <v>1186.48</v>
+        <v>753.92</v>
       </c>
       <c r="F30" s="8">
         <f>D30*E30</f>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="G30" s="12" t="inlineStr">
         <is>
-          <t>Fourniture Octet Plus devis DE044128 du 15/10/2026 (ZVK EasyLan, garantie système 25 ans ; baies LIEN'K), par annexe : coffret IP55 12U + bandeau (432.56 €) + liaison OS2 12 brins ≈ 150 ml avec tiroirs, fusion, tests (753.92 €) = 1186.48 €. Switch fourni par EXYTE.</t>
+          <t>Fourniture Octet Plus devis DE044128 du 15/10/2026 (ZVK EasyLan, garantie système 25 ans ; baies LIEN'K), par annexe : liaison OS2 12 brins ≈ 150 ml avec tiroir, fusion, tests = 753.92 €. Coffret IP55 fourni et posé par SPIE (retiré du devis Octet Plus). Switch fourni par EXYTE.</t>
         </is>
       </c>
     </row>

</xml_diff>